<commit_message>
New crime data collected
</commit_message>
<xml_diff>
--- a/data/source/weekly/cs-en-us-001pct.xlsx
+++ b/data/source/weekly/cs-en-us-001pct.xlsx
@@ -69,7 +69,7 @@
         <family val="2"/>
         <rFont val="Andale WT"/>
       </rPr>
-      <t xml:space="preserve">6</t>
+      <t xml:space="preserve">7</t>
     </r>
   </si>
   <si>
@@ -95,7 +95,7 @@
         <family val="2"/>
         <rFont val="Andale WT"/>
       </rPr>
-      <t xml:space="preserve">2/2/2026</t>
+      <t xml:space="preserve">2/9/2026</t>
     </r>
     <r>
       <rPr>
@@ -113,7 +113,7 @@
         <family val="2"/>
         <rFont val="Andale WT"/>
       </rPr>
-      <t xml:space="preserve">2/8/2026</t>
+      <t xml:space="preserve">2/15/2026</t>
     </r>
   </si>
   <si>
@@ -895,11 +895,11 @@
       <c r="C15" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="15">
-        <v>3</v>
-      </c>
-      <c r="E15" s="14">
-        <v>-100</v>
+      <c r="D15" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>21</v>
       </c>
       <c r="F15" s="13" t="s">
         <v>20</v>
@@ -934,40 +934,40 @@
         <v>23</v>
       </c>
       <c r="C16" s="15">
+        <v>1</v>
+      </c>
+      <c r="D16" s="15">
         <v>2</v>
       </c>
-      <c r="D16" s="15">
-        <v>5</v>
-      </c>
       <c r="E16" s="14">
-        <v>-60</v>
+        <v>-50</v>
       </c>
       <c r="F16" s="15">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G16" s="15">
         <v>8</v>
       </c>
       <c r="H16" s="14">
-        <v>12.5</v>
+        <v>-12.5</v>
       </c>
       <c r="I16" s="15">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J16" s="15">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K16" s="14">
-        <v>63.636363636363</v>
+        <v>46.153846153846</v>
       </c>
       <c r="L16" s="14">
-        <v>20</v>
+        <v>11.764705882352</v>
       </c>
       <c r="M16" s="14">
-        <v>125</v>
+        <v>137.5</v>
       </c>
       <c r="N16" s="14">
-        <v>-81.443298969072</v>
+        <v>-84.297520661157</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -984,31 +984,31 @@
         <v>100</v>
       </c>
       <c r="F17" s="15">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G17" s="15">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H17" s="14">
-        <v>37.5</v>
+        <v>100</v>
       </c>
       <c r="I17" s="15">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="J17" s="15">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K17" s="14">
-        <v>162.5</v>
+        <v>160</v>
       </c>
       <c r="L17" s="14">
-        <v>110</v>
+        <v>85.714285714285</v>
       </c>
       <c r="M17" s="14">
-        <v>200</v>
+        <v>188.888888888889</v>
       </c>
       <c r="N17" s="14">
-        <v>31.25</v>
+        <v>36.842105263157</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -1019,37 +1019,37 @@
         <v>1</v>
       </c>
       <c r="D18" s="15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E18" s="14">
-        <v>-83.333333333333</v>
+        <v>-66.666666666666</v>
       </c>
       <c r="F18" s="15">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G18" s="15">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H18" s="14">
-        <v>-50</v>
+        <v>-58.823529411764</v>
       </c>
       <c r="I18" s="15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J18" s="15">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K18" s="14">
-        <v>-31.578947368421</v>
+        <v>-36.363636363636</v>
       </c>
       <c r="L18" s="14">
-        <v>-40.909090909090</v>
+        <v>-46.153846153846</v>
       </c>
       <c r="M18" s="14">
-        <v>-40.909090909090</v>
+        <v>-44</v>
       </c>
       <c r="N18" s="14">
-        <v>-86.458333333333</v>
+        <v>-86.538461538461</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -1057,40 +1057,40 @@
         <v>26</v>
       </c>
       <c r="C19" s="15">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D19" s="15">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E19" s="14">
-        <v>-10.714285714285</v>
+        <v>-27.272727272727</v>
       </c>
       <c r="F19" s="15">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G19" s="15">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="H19" s="14">
-        <v>3.260869565217</v>
+        <v>-6</v>
       </c>
       <c r="I19" s="15">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="J19" s="15">
-        <v>123</v>
+        <v>156</v>
       </c>
       <c r="K19" s="14">
-        <v>5.691056910569</v>
+        <v>-1.282051282051</v>
       </c>
       <c r="L19" s="14">
-        <v>30</v>
+        <v>25.203252032520</v>
       </c>
       <c r="M19" s="14">
-        <v>17.117117117117</v>
+        <v>15.789473684210</v>
       </c>
       <c r="N19" s="14">
-        <v>-65.053763440860</v>
+        <v>-64.018691588785</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -1098,40 +1098,40 @@
         <v>27</v>
       </c>
       <c r="C20" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="15">
         <v>1</v>
       </c>
       <c r="E20" s="14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F20" s="15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G20" s="15">
         <v>2</v>
       </c>
       <c r="H20" s="14">
-        <v>-50</v>
+        <v>50</v>
       </c>
       <c r="I20" s="15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J20" s="15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="14">
-        <v>0</v>
+        <v>33.333333333333</v>
       </c>
       <c r="L20" s="14">
-        <v>-33.333333333333</v>
-      </c>
-      <c r="M20" s="13" t="s">
-        <v>21</v>
+        <v>33.333333333333</v>
+      </c>
+      <c r="M20" s="14">
+        <v>100</v>
       </c>
       <c r="N20" s="14">
-        <v>-98.130841121495</v>
+        <v>-96.774193548387</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -1139,78 +1139,78 @@
         <v>28</v>
       </c>
       <c r="C21" s="17">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D21" s="17">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E21" s="18">
-        <v>-26.666666666666</v>
+        <v>-21.951219512195</v>
       </c>
       <c r="F21" s="17">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G21" s="17">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="H21" s="18">
-        <v>-3.875968992248</v>
+        <v>-8.759124087591</v>
       </c>
       <c r="I21" s="17">
-        <v>184</v>
+        <v>217</v>
       </c>
       <c r="J21" s="17">
-        <v>168</v>
+        <v>209</v>
       </c>
       <c r="K21" s="18">
-        <v>9.523809523809</v>
+        <v>3.827751196172</v>
       </c>
       <c r="L21" s="18">
-        <v>20.261437908496</v>
+        <v>15.425531914893</v>
       </c>
       <c r="M21" s="18">
-        <v>24.324324324324</v>
+        <v>22.598870056497</v>
       </c>
       <c r="N21" s="18">
-        <v>-73.294629898403</v>
+        <v>-72.772898368883</v>
       </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="13" t="s">
-        <v>20</v>
+      <c r="C22" s="15">
+        <v>1</v>
       </c>
       <c r="D22" s="15">
         <v>3</v>
       </c>
       <c r="E22" s="14">
-        <v>-100</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>20</v>
+        <v>-66.666666666666</v>
+      </c>
+      <c r="F22" s="15">
+        <v>1</v>
       </c>
       <c r="G22" s="15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H22" s="14">
-        <v>-100</v>
+        <v>-87.5</v>
       </c>
       <c r="I22" s="15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J22" s="15">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K22" s="14">
-        <v>-71.428571428571</v>
+        <v>-70</v>
       </c>
       <c r="L22" s="14">
-        <v>-66.666666666666</v>
+        <v>-62.5</v>
       </c>
       <c r="M22" s="14">
-        <v>-80</v>
+        <v>-75</v>
       </c>
       <c r="N22" s="13" t="s">
         <v>21</v>
@@ -1262,37 +1262,37 @@
         <v>31</v>
       </c>
       <c r="C24" s="15">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D24" s="15">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E24" s="14">
-        <v>-27.941176470588</v>
+        <v>-31.506849315068</v>
       </c>
       <c r="F24" s="15">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="G24" s="15">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="H24" s="14">
-        <v>-28.413284132841</v>
+        <v>-29.924242424242</v>
       </c>
       <c r="I24" s="15">
-        <v>289</v>
+        <v>339</v>
       </c>
       <c r="J24" s="15">
-        <v>368</v>
+        <v>441</v>
       </c>
       <c r="K24" s="14">
-        <v>-21.467391304347</v>
+        <v>-23.129251700680</v>
       </c>
       <c r="L24" s="14">
-        <v>-30.528846153846</v>
+        <v>-30.816326530612</v>
       </c>
       <c r="M24" s="14">
-        <v>80.625</v>
+        <v>88.333333333333</v>
       </c>
       <c r="N24" s="13" t="s">
         <v>21</v>
@@ -1303,34 +1303,34 @@
         <v>32</v>
       </c>
       <c r="C25" s="15">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D25" s="15">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="E25" s="14">
-        <v>-31.428571428571</v>
+        <v>-37.179487179487</v>
       </c>
       <c r="F25" s="15">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="G25" s="15">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="H25" s="14">
-        <v>-24.528301886792</v>
+        <v>-30.597014925373</v>
       </c>
       <c r="I25" s="15">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="J25" s="15">
-        <v>362</v>
+        <v>440</v>
       </c>
       <c r="K25" s="14">
-        <v>-17.403314917127</v>
+        <v>-20.681818181818</v>
       </c>
       <c r="L25" s="14">
-        <v>-27.602905569007</v>
+        <v>-28.629856850715</v>
       </c>
       <c r="M25" s="13" t="s">
         <v>21</v>
@@ -1344,37 +1344,37 @@
         <v>33</v>
       </c>
       <c r="C26" s="15">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D26" s="15">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E26" s="14">
-        <v>16.666666666666</v>
+        <v>-20</v>
       </c>
       <c r="F26" s="15">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G26" s="15">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H26" s="14">
-        <v>-42.857142857142</v>
+        <v>-27.027027027027</v>
       </c>
       <c r="I26" s="15">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="J26" s="15">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="K26" s="14">
-        <v>-34.693877551020</v>
+        <v>-33.898305084745</v>
       </c>
       <c r="L26" s="14">
-        <v>6.666666666666</v>
+        <v>-15.217391304347</v>
       </c>
       <c r="M26" s="14">
-        <v>33.333333333333</v>
+        <v>34.482758620689</v>
       </c>
       <c r="N26" s="13" t="s">
         <v>21</v>
@@ -1387,11 +1387,11 @@
       <c r="C27" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="15">
-        <v>3</v>
-      </c>
-      <c r="E27" s="14">
-        <v>-100</v>
+      <c r="D27" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>21</v>
       </c>
       <c r="F27" s="13" t="s">
         <v>20</v>
@@ -1426,34 +1426,34 @@
         <v>35</v>
       </c>
       <c r="C28" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E28" s="14">
-        <v>-66.666666666666</v>
+        <v>0</v>
       </c>
       <c r="F28" s="15">
         <v>4</v>
       </c>
       <c r="G28" s="15">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H28" s="14">
-        <v>-20</v>
+        <v>-42.857142857142</v>
       </c>
       <c r="I28" s="15">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J28" s="15">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K28" s="14">
-        <v>80</v>
+        <v>42.857142857142</v>
       </c>
       <c r="L28" s="14">
-        <v>0</v>
+        <v>11.111111111111</v>
       </c>
       <c r="M28" s="13" t="s">
         <v>21</v>
@@ -1566,14 +1566,14 @@
       <c r="H31" s="14">
         <v>-100</v>
       </c>
-      <c r="I31" s="13" t="s">
-        <v>20</v>
+      <c r="I31" s="15">
+        <v>1</v>
       </c>
       <c r="J31" s="15">
         <v>2</v>
       </c>
       <c r="K31" s="14">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="L31" s="13" t="s">
         <v>21</v>

</xml_diff>